<commit_message>
PREDIMIN v5: red neuronal en ensamble, validacion agrupada por fecha y revision del plan de tesis
- Red neuronal: ensamble de 10 MLP con bootstrap, objetivo log(1+PM10), L-BFGS,
  arquitectura por optimizacion bayesiana; compite tambien en clasificacion
- Analisis detallado de la red (arquitectura, regularizacion, curva de
  aprendizaje, ROC, importancia por permutacion) y segunda opinion en la app
- Division 80:20 y validacion cruzada agrupadas por fecha (evita fuga de datos)
- docs/REVISION_PLAN_TESIS.md: observaciones al plan y textos propuestos
- Resultados regenerados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012GiUc3yWWkbUsXoVxUQVw8
</commit_message>
<xml_diff>
--- a/outputs/RESULTADOS_TESIS.xlsx
+++ b/outputs/RESULTADOS_TESIS.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_Depuracion" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_Descriptivos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_Correlaciones" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_Modelos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_Clasificacion" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_Importancia_SHAP" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7_Escenarios" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8_Hiperparametros" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="1_Depuracion" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2_Descriptivos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="3_Correlaciones" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="4_Modelos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="5_Clasificacion" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="6_Importancia_SHAP" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="7_Escenarios" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="8_Hiperparametros" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="9_Red_Neuronal" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="10_RN_Importancia" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -516,6 +518,408 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>variable</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>perdida_R2_regresion</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>perdida_AUC_clasificacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Humedad relativa (%)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>humedad_relativa_pct</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.6141</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.178</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Hora del disparo</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>hora</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.2778</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.0718</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Direccion del viento (coseno)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>viento_cos</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.0447</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.06279999999999999</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Mes (seno)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>mes_sin</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.0658</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.0131</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ANFO (kg)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>anfo_kg</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.0263</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.0102</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Velocidad del viento (m/s)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>velocidad_viento_ms</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.3372</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Retardo entre filas (ms)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>tiempo_fila_ms</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.0226</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.008800000000000001</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Indice seco</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>indice_seco</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.0618</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.008200000000000001</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Disparos en el dia</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>n_eventos</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.1078</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.0047</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Precipitacion (mm)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>precipitacion_mm</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.0007</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.0028</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Fraccion de emulsion</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>fraccion_emulsion</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.1023</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-0.0038</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Explosivo por taladro (kg)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>explosivo_por_taladro</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.0728</v>
+      </c>
+      <c r="D13" t="n">
+        <v>-0.0038</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Tonelaje fracturado (t)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>tonelaje_tm</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.0624</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-0.0044</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Explosivo total - Heavy ANFO (kg)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>explosivo_total_kg</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.1069</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-0.0057</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Numero de taladros</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>numero_taladros</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.1163</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-0.0068</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Mes (coseno)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>mes_cos</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.0119</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-0.0073</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Emulsion (kg)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>emulsion_kg</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.1716</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-0.0076</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Direccion del viento (seno)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>viento_sin</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.0619</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-0.0154</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Factor de carga (kg/t)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>factor_carga_kg_t</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.0017</v>
+      </c>
+      <c r="D20" t="n">
+        <v>-0.017</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Retardo entre taladros (ms)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>tiempo_taladro_ms</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>-0.0107</v>
+      </c>
+      <c r="D21" t="n">
+        <v>-0.031</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -1847,28 +2251,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.2176</v>
+        <v>0.2164</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1039</v>
+        <v>0.1102</v>
       </c>
       <c r="D2" t="n">
-        <v>30.164</v>
+        <v>32.6516</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2342</v>
+        <v>0.2539</v>
       </c>
       <c r="F2" t="n">
-        <v>36.7257</v>
+        <v>25.8966</v>
       </c>
       <c r="G2" t="n">
-        <v>21.344</v>
+        <v>17.4594</v>
       </c>
       <c r="H2" t="n">
-        <v>108.73</v>
+        <v>106.6</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0315</v>
+        <v>0.0344</v>
       </c>
     </row>
     <row r="3">
@@ -1878,141 +2282,141 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1871</v>
+        <v>0.1951</v>
       </c>
       <c r="C3" t="n">
-        <v>0.07870000000000001</v>
+        <v>0.0688</v>
       </c>
       <c r="D3" t="n">
-        <v>30.7145</v>
+        <v>33.2719</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2003</v>
+        <v>0.2118</v>
       </c>
       <c r="F3" t="n">
-        <v>37.5303</v>
+        <v>26.6179</v>
       </c>
       <c r="G3" t="n">
-        <v>21.3204</v>
+        <v>17.5317</v>
       </c>
       <c r="H3" t="n">
-        <v>109.99</v>
+        <v>112.33</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1807</v>
+        <v>0.1921</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0917</v>
+        <v>0.0785</v>
       </c>
       <c r="D4" t="n">
-        <v>30.8211</v>
+        <v>33.2615</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2044</v>
+        <v>0.2018</v>
       </c>
       <c r="F4" t="n">
-        <v>37.4337</v>
+        <v>26.7849</v>
       </c>
       <c r="G4" t="n">
-        <v>21.1455</v>
+        <v>18.2712</v>
       </c>
       <c r="H4" t="n">
-        <v>106.64</v>
+        <v>115.66</v>
       </c>
       <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.1715</v>
+        <v>0.1828</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1018</v>
+        <v>0.1135</v>
       </c>
       <c r="D5" t="n">
-        <v>30.9379</v>
+        <v>33.3484</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2191</v>
+        <v>0.16</v>
       </c>
       <c r="F5" t="n">
-        <v>37.0855</v>
+        <v>27.4775</v>
       </c>
       <c r="G5" t="n">
-        <v>21.3595</v>
+        <v>18.2281</v>
       </c>
       <c r="H5" t="n">
-        <v>109.31</v>
+        <v>112.55</v>
       </c>
       <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.1701</v>
+        <v>0.1797</v>
       </c>
       <c r="C6" t="n">
-        <v>0.1015</v>
+        <v>0.07779999999999999</v>
       </c>
       <c r="D6" t="n">
-        <v>31.0189</v>
+        <v>33.569</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1892</v>
+        <v>0.2158</v>
       </c>
       <c r="F6" t="n">
-        <v>37.789</v>
+        <v>26.5493</v>
       </c>
       <c r="G6" t="n">
-        <v>21.699</v>
+        <v>18.0236</v>
       </c>
       <c r="H6" t="n">
-        <v>116.12</v>
+        <v>118.96</v>
       </c>
       <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.1635</v>
+        <v>0.1674</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0859</v>
+        <v>0.0774</v>
       </c>
       <c r="D7" t="n">
-        <v>31.1478</v>
+        <v>33.7789</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1999</v>
+        <v>0.2368</v>
       </c>
       <c r="F7" t="n">
-        <v>37.5395</v>
+        <v>26.1923</v>
       </c>
       <c r="G7" t="n">
-        <v>21.8601</v>
+        <v>17.9174</v>
       </c>
       <c r="H7" t="n">
-        <v>118.6</v>
+        <v>115.92</v>
       </c>
       <c r="I7" t="inlineStr"/>
     </row>
@@ -2023,25 +2427,25 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.0856</v>
+        <v>0.1294</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0765</v>
+        <v>0.1235</v>
       </c>
       <c r="D8" t="n">
-        <v>32.5802</v>
+        <v>34.3659</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.041</v>
+        <v>0.2037</v>
       </c>
       <c r="F8" t="n">
-        <v>42.8196</v>
+        <v>26.7538</v>
       </c>
       <c r="G8" t="n">
-        <v>22.7743</v>
+        <v>16.7321</v>
       </c>
       <c r="H8" t="n">
-        <v>66.84999999999999</v>
+        <v>81.65000000000001</v>
       </c>
       <c r="I8" t="inlineStr"/>
     </row>
@@ -2056,7 +2460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2106,107 +2510,129 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8133</v>
+        <v>0.801</v>
       </c>
       <c r="C2" t="n">
-        <v>0.7941</v>
+        <v>0.76</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7647</v>
+        <v>0.6923</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5417</v>
+        <v>0.4091</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6341</v>
+        <v>0.5143</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.8061</v>
+        <v>0.7953</v>
       </c>
       <c r="C3" t="n">
-        <v>0.796</v>
+        <v>0.7784</v>
       </c>
       <c r="D3" t="n">
-        <v>0.4118</v>
+        <v>0.6923</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5</v>
+        <v>0.45</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4516</v>
+        <v>0.5455</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.8038999999999999</v>
+        <v>0.7911</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7518</v>
+        <v>0.791</v>
       </c>
       <c r="D4" t="n">
-        <v>0.4118</v>
+        <v>0.5385</v>
       </c>
       <c r="E4" t="n">
-        <v>0.5385</v>
+        <v>0.5</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4667</v>
+        <v>0.5185</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LightGBM</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.7958</v>
+        <v>0.7899</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7381</v>
+        <v>0.7819</v>
       </c>
       <c r="D5" t="n">
-        <v>0.4118</v>
+        <v>0.3846</v>
       </c>
       <c r="E5" t="n">
-        <v>0.35</v>
+        <v>0.4167</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3784</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RedNeuronal_MLP</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.7575</v>
+        <v>0.7887</v>
       </c>
       <c r="C6" t="n">
-        <v>0.7858000000000001</v>
+        <v>0.7899</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1765</v>
+        <v>0.4615</v>
       </c>
       <c r="E6" t="n">
-        <v>0.375</v>
+        <v>0.5455</v>
       </c>
       <c r="F6" t="n">
-        <v>0.24</v>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LightGBM</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.7747000000000001</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.7956</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.4615</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.3529</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.4</v>
       </c>
     </row>
   </sheetData>
@@ -2257,277 +2683,277 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.4511</v>
+        <v>8.193300000000001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Direccion del viento (coseno)</t>
+          <t>Mes (seno)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>viento_cos</t>
+          <t>mes_sin</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3.1014</v>
+        <v>4.2218</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mes (seno)</t>
+          <t>Direccion del viento (coseno)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>mes_sin</t>
+          <t>viento_cos</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2.9363</v>
+        <v>2.4191</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Indice seco</t>
+          <t>Mes (coseno)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>indice_seco</t>
+          <t>mes_cos</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2.4142</v>
+        <v>2.0885</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Fraccion de emulsion</t>
+          <t>Indice seco</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>fraccion_emulsion</t>
+          <t>indice_seco</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.5711</v>
+        <v>2.034</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Mes (coseno)</t>
+          <t>Fraccion de emulsion</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>mes_cos</t>
+          <t>fraccion_emulsion</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.5122</v>
+        <v>1.6182</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Hora del disparo</t>
+          <t>Direccion del viento (seno)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>viento_sin</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1.0817</v>
+        <v>1.5102</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Direccion del viento (seno)</t>
+          <t>Hora del disparo</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>viento_sin</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.9594</v>
+        <v>1.2344</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ANFO (kg)</t>
+          <t>Retardo entre filas (ms)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>anfo_kg</t>
+          <t>tiempo_fila_ms</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.5251</v>
+        <v>0.4824</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Velocidad del viento (m/s)</t>
+          <t>Retardo entre taladros (ms)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>velocidad_viento_ms</t>
+          <t>tiempo_taladro_ms</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.5098</v>
+        <v>0.3923</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Explosivo por taladro (kg)</t>
+          <t>Velocidad del viento (m/s)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>explosivo_por_taladro</t>
+          <t>velocidad_viento_ms</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.3367</v>
+        <v>0.3868</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Retardo entre taladros (ms)</t>
+          <t>ANFO (kg)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>tiempo_taladro_ms</t>
+          <t>anfo_kg</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.3119</v>
+        <v>0.3166</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Retardo entre filas (ms)</t>
+          <t>Factor de carga (kg/t)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>tiempo_fila_ms</t>
+          <t>factor_carga_kg_t</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.2666</v>
+        <v>0.2975</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Disparos en el dia</t>
+          <t>Tonelaje fracturado (t)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>n_eventos</t>
+          <t>tonelaje_tm</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.2194</v>
+        <v>0.2962</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Explosivo total - Heavy ANFO (kg)</t>
+          <t>Disparos en el dia</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>explosivo_total_kg</t>
+          <t>n_eventos</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.2124</v>
+        <v>0.2523</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Numero de taladros</t>
+          <t>Explosivo por taladro (kg)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>numero_taladros</t>
+          <t>explosivo_por_taladro</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.1924</v>
+        <v>0.2333</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Emulsion (kg)</t>
+          <t>Explosivo total - Heavy ANFO (kg)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>emulsion_kg</t>
+          <t>explosivo_total_kg</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.1869</v>
+        <v>0.2038</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Tonelaje fracturado (t)</t>
+          <t>Numero de taladros</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>tonelaje_tm</t>
+          <t>numero_taladros</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.1683</v>
+        <v>0.199</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Factor de carga (kg/t)</t>
+          <t>Emulsion (kg)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>factor_carga_kg_t</t>
+          <t>emulsion_kg</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.1626</v>
+        <v>0.1813</v>
       </c>
     </row>
     <row r="21">
@@ -2542,7 +2968,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.1039</v>
+        <v>0.1208</v>
       </c>
     </row>
   </sheetData>
@@ -2600,14 +3026,14 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>49.9</v>
+        <v>45</v>
       </c>
       <c r="C2" t="n">
-        <v>0.674</v>
+        <v>0.624</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NARANJA</t>
+          <t>AMARILLO</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -2624,7 +3050,7 @@
         <v>46.8</v>
       </c>
       <c r="C3" t="n">
-        <v>0.643</v>
+        <v>0.616</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -2632,7 +3058,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>6.2</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="4">
@@ -2642,10 +3068,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>47.3</v>
+        <v>50.2</v>
       </c>
       <c r="C4" t="n">
-        <v>0.649</v>
+        <v>0.653</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -2653,7 +3079,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>5.2</v>
+        <v>-11.6</v>
       </c>
     </row>
     <row r="5">
@@ -2663,10 +3089,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>52.8</v>
+        <v>49.4</v>
       </c>
       <c r="C5" t="n">
-        <v>0.698</v>
+        <v>0.657</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -2674,7 +3100,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>-5.8</v>
+        <v>-9.800000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -2684,18 +3110,18 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>49.2</v>
+        <v>44.9</v>
       </c>
       <c r="C6" t="n">
-        <v>0.634</v>
+        <v>0.602</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NARANJA</t>
+          <t>AMARILLO</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>1.4</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="7">
@@ -2705,10 +3131,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>38.5</v>
+        <v>36.4</v>
       </c>
       <c r="C7" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.512</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -2716,7 +3142,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>22.8</v>
+        <v>19.1</v>
       </c>
     </row>
     <row r="8">
@@ -2726,18 +3152,18 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>43.1</v>
+        <v>45.2</v>
       </c>
       <c r="C8" t="n">
-        <v>0.464</v>
+        <v>0.443</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>AMARILLO</t>
+          <t>NARANJA</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>13.6</v>
+        <v>-0.4</v>
       </c>
     </row>
   </sheetData>
@@ -2778,7 +3204,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{"n_estimators": 550, "max_depth": 19, "min_samples_leaf": 8, "max_features": 0.38211092558820536}</t>
+          <t>{"n_estimators": 200, "max_depth": 7, "min_samples_leaf": 7, "max_features": 0.62658035888649}</t>
         </is>
       </c>
     </row>
@@ -2790,7 +3216,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"n_estimators": 150, "max_depth": 15, "min_samples_leaf": 5, "max_features": 0.7087738489021961}</t>
+          <t>{"n_estimators": 400, "max_depth": 9, "min_samples_leaf": 4, "max_features": 0.9768535915448162}</t>
         </is>
       </c>
     </row>
@@ -2802,7 +3228,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"n_estimators": 100, "learning_rate": 0.011381659820186149, "max_depth": 3, "min_samples_leaf": 7, "subsample": 0.7447664874619755}</t>
+          <t>{"n_estimators": 100, "learning_rate": 0.017253254730863327, "max_depth": 4, "min_samples_leaf": 10, "subsample": 0.6268494210878071}</t>
         </is>
       </c>
     </row>
@@ -2814,7 +3240,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"n_estimators": 100, "learning_rate": 0.01529685107334084, "max_depth": 2, "subsample": 0.8189736931888547, "colsample_bytree": 0.8275765985657748, "min_child_weight": 7.363911420084752, "reg_lambda": 0.003412485917285091}</t>
+          <t>{"n_estimators": 200, "learning_rate": 0.016286716884536492, "max_depth": 2, "subsample": 0.9116822556022266, "colsample_bytree": 0.7740471563755147, "min_child_weight": 7.83920207271774, "reg_lambda": 0.08241886448735286}</t>
         </is>
       </c>
     </row>
@@ -2826,7 +3252,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"n_estimators": 100, "learning_rate": 0.017076054474389826, "num_leaves": 35, "min_child_samples": 29, "subsample": 0.7284727804886667, "subsample_freq": 1, "colsample_bytree": 0.8262498898771143, "reg_lambda": 0.019166122961542877}</t>
+          <t>{"n_estimators": 100, "learning_rate": 0.02645373036172781, "num_leaves": 38, "min_child_samples": 29, "subsample": 0.7997688291894813, "subsample_freq": 1, "colsample_bytree": 0.6224884932836999, "reg_lambda": 0.005550202088313911}</t>
         </is>
       </c>
     </row>
@@ -2838,7 +3264,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"iterations": 300, "learning_rate": 0.015521231712211063, "depth": 3, "l2_leaf_reg": 7.482569693397399}</t>
+          <t>{"iterations": 500, "learning_rate": 0.03553023643604902, "depth": 8, "l2_leaf_reg": 1.46442172093703}</t>
         </is>
       </c>
     </row>
@@ -2850,8 +3276,397 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"n_capas": 1, "neuronas": 64, "alpha": 21.04998058047481, "learning_rate_init": 0.004138040112561018}</t>
-        </is>
+          <t>{"n_capas": 1, "neuronas": 4, "activacion": "tanh", "alpha": 2.1741399821159484}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Seccion</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Indicador</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>entradas</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>capas_ocultas</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>[4]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>activacion</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>tanh</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>salida</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>optimizador</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>L-BFGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>regularizacion_L2_alpha</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2.174139982115948</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>redes_en_ensamble</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>parametros_por_red</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>objetivo_regresion</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>log(1 + PM10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>regresion</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>R2_CV_medio</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.1294</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>regresion</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>R2_CV_desv</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.1235</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>regresion</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>R2_test</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.2037</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>regresion</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>RMSE_test</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>26.7538</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>regresion</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>MAE_test</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>16.7321</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>regresion</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>MAPE_%_test</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>81.65000000000001</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>regresion</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>cobertura_intervalo_90_%</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>regresion</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ancho_medio_intervalo_ugm3</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>36.86</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>clasificacion</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>AUC_CV</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.7887</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>clasificacion</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>AUC_CV_desv</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.0698</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>clasificacion</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>AUC_test</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0.7899</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>clasificacion</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Sensibilidad_test</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>0.4615</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>clasificacion</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Precision_test</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0.5455</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>clasificacion</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>F1_test</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rediseño profesional de la aplicación web
- Encabezado institucional, tarjetas de indicadores y alerta con icono y etiqueta
- Gráficos interactivos (Plotly): PM10 frente a OMS/ECA con rango de la red
  neuronal, contribuciones SHAP, escenarios y comparación de modelos
- Nueva pestaña 'Acerca del sistema' (flujo, niveles de alerta, limitaciones, equipo)
- Tema visual (.streamlit/config.toml), resultados en vivo sin botón
- Etiquetas de variables centralizadas en config.py y textos con tildes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012GiUc3yWWkbUsXoVxUQVw8
</commit_message>
<xml_diff>
--- a/outputs/RESULTADOS_TESIS.xlsx
+++ b/outputs/RESULTADOS_TESIS.xlsx
@@ -594,7 +594,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Direccion del viento (coseno)</t>
+          <t>Dirección del viento (coseno)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -684,7 +684,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Indice seco</t>
+          <t>Índice seco</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -702,7 +702,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Disparos en el dia</t>
+          <t>Disparos en el día</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -720,7 +720,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Precipitacion (mm)</t>
+          <t>Precipitación (mm)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -738,7 +738,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Fraccion de emulsion</t>
+          <t>Fracción de emulsión</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -810,7 +810,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Numero de taladros</t>
+          <t>Número de taladros</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -846,7 +846,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Emulsion (kg)</t>
+          <t>Emulsión (kg)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -864,7 +864,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Direccion del viento (seno)</t>
+          <t>Dirección del viento (seno)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -990,7 +990,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Numero de taladros</t>
+          <t>Número de taladros</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1083,7 +1083,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Emulsion (kg)</t>
+          <t>Emulsión (kg)</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -1145,7 +1145,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Disparos en el dia</t>
+          <t>Disparos en el día</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -1300,7 +1300,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Precipitacion (mm)</t>
+          <t>Precipitación (mm)</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -1362,7 +1362,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Direccion del viento (seno)</t>
+          <t>Dirección del viento (seno)</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1393,7 +1393,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Direccion del viento (coseno)</t>
+          <t>Dirección del viento (coseno)</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1548,7 +1548,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Fraccion de emulsion</t>
+          <t>Fracción de emulsión</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1579,7 +1579,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Indice seco</t>
+          <t>Índice seco</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1610,7 +1610,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PM10 (ug/m3)</t>
+          <t>PM10 (µg/m³)</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1767,7 +1767,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Indice seco</t>
+          <t>Índice seco</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1791,7 +1791,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Precipitacion (mm)</t>
+          <t>Precipitación (mm)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1815,7 +1815,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Direccion del viento (coseno)</t>
+          <t>Dirección del viento (coseno)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1839,7 +1839,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Fraccion de emulsion</t>
+          <t>Fracción de emulsión</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1935,7 +1935,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Emulsion (kg)</t>
+          <t>Emulsión (kg)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2007,7 +2007,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Numero de taladros</t>
+          <t>Número de taladros</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2079,7 +2079,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Direccion del viento (seno)</t>
+          <t>Dirección del viento (seno)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2151,7 +2151,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Disparos en el dia</t>
+          <t>Disparos en el día</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2704,7 +2704,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Direccion del viento (coseno)</t>
+          <t>Dirección del viento (coseno)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2734,7 +2734,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Indice seco</t>
+          <t>Índice seco</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2749,7 +2749,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Fraccion de emulsion</t>
+          <t>Fracción de emulsión</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2764,7 +2764,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Direccion del viento (seno)</t>
+          <t>Dirección del viento (seno)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2884,7 +2884,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Disparos en el dia</t>
+          <t>Disparos en el día</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2929,7 +2929,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Numero de taladros</t>
+          <t>Número de taladros</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2944,7 +2944,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Emulsion (kg)</t>
+          <t>Emulsión (kg)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2959,7 +2959,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Precipitacion (mm)</t>
+          <t>Precipitación (mm)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3085,7 +3085,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Un solo disparo en el dia</t>
+          <t>Un solo disparo en el día</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -3127,7 +3127,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Condicion mas humeda (+15 % HR)</t>
+          <t>Condición más húmeda (+15 % HR)</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -3148,7 +3148,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Viento calmo (0.5 m/s)</t>
+          <t>Viento calmo (0,5 m/s)</t>
         </is>
       </c>
       <c r="B8" t="n">

</xml_diff>